<commit_message>
test(fixtures): BOW-923 第三幕夹具按原型 Y 逐人数据重做 (#334)
夹具逐人取自原型 Y，不复制评语；本代身份统一加 bow-923-v3- 前缀，与上一代主键不重叠；两步生成串联，CI 实跑提取与生成并逐字节比对。
</commit_message>
<xml_diff>
--- a/tests/fixtures/bow-923/作品评审表.xlsx
+++ b/tests/fixtures/bow-923/作品评审表.xlsx
@@ -411,34 +411,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D2" s="3" t="str">
-        <x:v>bow-923-team-work-orbit</x:v>
+        <x:v>bow-923-v3-work-001</x:v>
       </x:c>
       <x:c r="E2" s="3" t="str">
-        <x:v>组队作品</x:v>
-      </x:c>
-      <x:c r="F2" s="3" t="str">
-        <x:v>轨道队（演示）</x:v>
-      </x:c>
+        <x:v>个人作品</x:v>
+      </x:c>
+      <x:c r="F2" s="3"/>
       <x:c r="G2" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H2" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I2" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J2" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="K2" s="3" t="str">
-        <x:v>p-yeqing</x:v>
+        <x:v>s-28</x:v>
       </x:c>
       <x:c r="L2" s="3" t="str">
-        <x:v>叶青（演示）</x:v>
+        <x:v>许致远（演示）</x:v>
       </x:c>
       <x:c r="M2" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N2" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -447,7 +445,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P2" s="3" t="str">
-        <x:v>演示重建：作品主流程完整，能说明一次方案取舍，并现场复现失败后的恢复步骤。</x:v>
+        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="48" customHeight="1">
@@ -461,32 +459,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D3" s="3" t="str">
-        <x:v>bow-923-work-002</x:v>
+        <x:v>bow-923-v3-work-002</x:v>
       </x:c>
       <x:c r="E3" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F3" s="3"/>
       <x:c r="G3" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H3" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I3" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J3" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>优先录取</x:v>
       </x:c>
       <x:c r="K3" s="3" t="str">
-        <x:v>p-yeqing</x:v>
+        <x:v>s-28</x:v>
       </x:c>
       <x:c r="L3" s="3" t="str">
-        <x:v>叶青（演示）</x:v>
+        <x:v>许致远（演示）</x:v>
       </x:c>
       <x:c r="M3" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N3" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -495,7 +493,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P3" s="3" t="str">
-        <x:v>演示重建：完成了最小主流程；评审时未充分展示边界场景，按原档位记录。</x:v>
+        <x:v>演示重建：作品主流程完整，能说明一次方案取舍，并现场复现失败后的恢复步骤。</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="48" customHeight="1">
@@ -509,34 +507,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D4" s="3" t="str">
-        <x:v>bow-923-team-work-orbit</x:v>
+        <x:v>bow-923-v3-work-003</x:v>
       </x:c>
       <x:c r="E4" s="3" t="str">
-        <x:v>组队作品</x:v>
-      </x:c>
-      <x:c r="F4" s="3" t="str">
-        <x:v>轨道队（演示）</x:v>
-      </x:c>
+        <x:v>个人作品</x:v>
+      </x:c>
+      <x:c r="F4" s="3"/>
       <x:c r="G4" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H4" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I4" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J4" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>优先录取</x:v>
       </x:c>
       <x:c r="K4" s="3" t="str">
-        <x:v>p-yeqing</x:v>
+        <x:v>s-28</x:v>
       </x:c>
       <x:c r="L4" s="3" t="str">
-        <x:v>叶青（演示）</x:v>
+        <x:v>许致远（演示）</x:v>
       </x:c>
       <x:c r="M4" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N4" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -559,32 +555,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D5" s="3" t="str">
-        <x:v>bow-923-work-004</x:v>
+        <x:v>bow-923-v3-work-004</x:v>
       </x:c>
       <x:c r="E5" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F5" s="3"/>
       <x:c r="G5" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H5" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I5" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J5" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="K5" s="3" t="str">
-        <x:v>p-yeqing</x:v>
+        <x:v>s-28</x:v>
       </x:c>
       <x:c r="L5" s="3" t="str">
-        <x:v>叶青（演示）</x:v>
+        <x:v>许致远（演示）</x:v>
       </x:c>
       <x:c r="M5" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N5" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -607,32 +603,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D6" s="3" t="str">
-        <x:v>bow-923-work-005</x:v>
+        <x:v>bow-923-v3-work-005</x:v>
       </x:c>
       <x:c r="E6" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F6" s="3"/>
       <x:c r="G6" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H6" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I6" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J6" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>优先录取</x:v>
       </x:c>
       <x:c r="K6" s="3" t="str">
-        <x:v>p-yeqing</x:v>
+        <x:v>s-28</x:v>
       </x:c>
       <x:c r="L6" s="3" t="str">
-        <x:v>叶青（演示）</x:v>
+        <x:v>许致远（演示）</x:v>
       </x:c>
       <x:c r="M6" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N6" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -655,23 +651,23 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D7" s="3" t="str">
-        <x:v>bow-923-work-006</x:v>
+        <x:v>bow-923-v3-work-006</x:v>
       </x:c>
       <x:c r="E7" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F7" s="3"/>
       <x:c r="G7" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H7" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I7" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J7" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>优先录取</x:v>
       </x:c>
       <x:c r="K7" s="3" t="str">
         <x:v>p-yeqing</x:v>
@@ -680,7 +676,7 @@
         <x:v>叶青（演示）</x:v>
       </x:c>
       <x:c r="M7" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N7" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -703,23 +699,23 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D8" s="3" t="str">
-        <x:v>bow-923-work-007</x:v>
+        <x:v>bow-923-v3-work-007</x:v>
       </x:c>
       <x:c r="E8" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F8" s="3"/>
       <x:c r="G8" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H8" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I8" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J8" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="K8" s="3" t="str">
         <x:v>p-yeqing</x:v>
@@ -728,7 +724,7 @@
         <x:v>叶青（演示）</x:v>
       </x:c>
       <x:c r="M8" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N8" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -737,7 +733,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P8" s="3" t="str">
-        <x:v>演示重建：作品主流程完整，能说明一次方案取舍，并现场复现失败后的恢复步骤。</x:v>
+        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="48" customHeight="1">
@@ -751,32 +747,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D9" s="3" t="str">
-        <x:v>bow-923-work-008</x:v>
+        <x:v>bow-923-v3-work-008</x:v>
       </x:c>
       <x:c r="E9" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F9" s="3"/>
       <x:c r="G9" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H9" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I9" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J9" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="K9" s="3" t="str">
-        <x:v>s-01</x:v>
+        <x:v>p-yeqing</x:v>
       </x:c>
       <x:c r="L9" s="3" t="str">
-        <x:v>任辞远（演示）</x:v>
+        <x:v>叶青（演示）</x:v>
       </x:c>
       <x:c r="M9" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N9" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -785,7 +781,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P9" s="3" t="str">
-        <x:v>演示重建：作品主流程完整，能说明一次方案取舍，并现场复现失败后的恢复步骤。</x:v>
+        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="48" customHeight="1">
@@ -799,32 +795,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D10" s="3" t="str">
-        <x:v>bow-923-work-009</x:v>
+        <x:v>bow-923-v3-work-009</x:v>
       </x:c>
       <x:c r="E10" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F10" s="3"/>
       <x:c r="G10" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H10" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="I10" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J10" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>刚过线</x:v>
       </x:c>
       <x:c r="K10" s="3" t="str">
-        <x:v>s-01</x:v>
+        <x:v>p-yeqing</x:v>
       </x:c>
       <x:c r="L10" s="3" t="str">
-        <x:v>任辞远（演示）</x:v>
+        <x:v>叶青（演示）</x:v>
       </x:c>
       <x:c r="M10" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N10" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -847,32 +843,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D11" s="3" t="str">
-        <x:v>bow-923-work-010</x:v>
+        <x:v>bow-923-v3-work-010</x:v>
       </x:c>
       <x:c r="E11" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F11" s="3"/>
       <x:c r="G11" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H11" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I11" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J11" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="K11" s="3" t="str">
-        <x:v>s-01</x:v>
+        <x:v>p-yeqing</x:v>
       </x:c>
       <x:c r="L11" s="3" t="str">
-        <x:v>任辞远（演示）</x:v>
+        <x:v>叶青（演示）</x:v>
       </x:c>
       <x:c r="M11" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N11" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -895,32 +891,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D12" s="3" t="str">
-        <x:v>bow-923-work-011</x:v>
+        <x:v>bow-923-v3-work-011</x:v>
       </x:c>
       <x:c r="E12" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F12" s="3"/>
       <x:c r="G12" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H12" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="I12" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J12" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>刚过线</x:v>
       </x:c>
       <x:c r="K12" s="3" t="str">
-        <x:v>s-01</x:v>
+        <x:v>p-yeqing</x:v>
       </x:c>
       <x:c r="L12" s="3" t="str">
-        <x:v>任辞远（演示）</x:v>
+        <x:v>叶青（演示）</x:v>
       </x:c>
       <x:c r="M12" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N12" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -929,7 +925,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P12" s="3" t="str">
-        <x:v>演示重建：作品主流程完整，能说明一次方案取舍，并现场复现失败后的恢复步骤。</x:v>
+        <x:v>演示重建：完成了最小主流程；评审时未充分展示边界场景，按原档位记录。</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="48" customHeight="1">
@@ -943,32 +939,34 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D13" s="3" t="str">
-        <x:v>bow-923-work-012</x:v>
+        <x:v>bow-923-v3-team-work-seven</x:v>
       </x:c>
       <x:c r="E13" s="3" t="str">
-        <x:v>个人作品</x:v>
-      </x:c>
-      <x:c r="F13" s="3"/>
+        <x:v>组队作品</x:v>
+      </x:c>
+      <x:c r="F13" s="3" t="str">
+        <x:v>七号队（演示）</x:v>
+      </x:c>
       <x:c r="G13" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H13" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I13" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="J13" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>优先录取</x:v>
       </x:c>
       <x:c r="K13" s="3" t="str">
-        <x:v>s-01</x:v>
+        <x:v>p-yeqing</x:v>
       </x:c>
       <x:c r="L13" s="3" t="str">
-        <x:v>任辞远（演示）</x:v>
+        <x:v>叶青（演示）</x:v>
       </x:c>
       <x:c r="M13" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N13" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -977,7 +975,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P13" s="3" t="str">
-        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
+        <x:v>演示重建：组队作品，三人分工完成整套流程，演示由队长主讲；按同队各自一行记录。</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="48" customHeight="1">
@@ -991,32 +989,34 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D14" s="3" t="str">
-        <x:v>bow-923-work-013</x:v>
+        <x:v>bow-923-v3-team-work-seven</x:v>
       </x:c>
       <x:c r="E14" s="3" t="str">
-        <x:v>个人作品</x:v>
-      </x:c>
-      <x:c r="F14" s="3"/>
+        <x:v>组队作品</x:v>
+      </x:c>
+      <x:c r="F14" s="3" t="str">
+        <x:v>七号队（演示）</x:v>
+      </x:c>
       <x:c r="G14" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H14" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I14" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="J14" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>优先录取</x:v>
       </x:c>
       <x:c r="K14" s="3" t="str">
-        <x:v>s-01</x:v>
+        <x:v>p-yeqing</x:v>
       </x:c>
       <x:c r="L14" s="3" t="str">
-        <x:v>任辞远（演示）</x:v>
+        <x:v>叶青（演示）</x:v>
       </x:c>
       <x:c r="M14" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N14" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -1025,7 +1025,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P14" s="3" t="str">
-        <x:v>演示重建：作品主流程完整，能说明一次方案取舍，并现场复现失败后的恢复步骤。</x:v>
+        <x:v>演示重建：组队作品，三人分工完成整套流程，演示由队长主讲；按同队各自一行记录。</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="48" customHeight="1">
@@ -1039,27 +1039,41 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D15" s="3" t="str">
-        <x:v>bow-923-work-014</x:v>
+        <x:v>bow-923-v3-work-014</x:v>
       </x:c>
       <x:c r="E15" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F15" s="3"/>
-      <x:c r="G15" s="3"/>
-      <x:c r="H15" s="3"/>
-      <x:c r="I15" s="3"/>
-      <x:c r="J15" s="3"/>
-      <x:c r="K15" s="3"/>
-      <x:c r="L15" s="3"/>
-      <x:c r="M15" s="10"/>
+      <x:c r="G15" s="3" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="H15" s="3" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I15" s="3" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="J15" s="3" t="str">
+        <x:v>刚过线</x:v>
+      </x:c>
+      <x:c r="K15" s="3" t="str">
+        <x:v>p-yeqing</x:v>
+      </x:c>
+      <x:c r="L15" s="3" t="str">
+        <x:v>叶青（演示）</x:v>
+      </x:c>
+      <x:c r="M15" s="10" t="n">
+        <x:v>46203.04166666667</x:v>
+      </x:c>
       <x:c r="N15" s="3" t="str">
         <x:v>xe-select-v1</x:v>
       </x:c>
       <x:c r="O15" s="3" t="str">
-        <x:v>缺段</x:v>
+        <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P15" s="3" t="str">
-        <x:v>演示重建：缺少入营选拔评审记录，未补造评价或评价人。</x:v>
+        <x:v>演示重建：完成了最小主流程；评审时未充分展示边界场景，按原档位记录。</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="48" customHeight="1">
@@ -1073,27 +1087,43 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D16" s="3" t="str">
-        <x:v>bow-923-work-015</x:v>
+        <x:v>bow-923-v3-team-work-seven</x:v>
       </x:c>
       <x:c r="E16" s="3" t="str">
-        <x:v>个人作品</x:v>
-      </x:c>
-      <x:c r="F16" s="3"/>
-      <x:c r="G16" s="3"/>
-      <x:c r="H16" s="3"/>
-      <x:c r="I16" s="3"/>
-      <x:c r="J16" s="3"/>
-      <x:c r="K16" s="3"/>
-      <x:c r="L16" s="3"/>
-      <x:c r="M16" s="10"/>
+        <x:v>组队作品</x:v>
+      </x:c>
+      <x:c r="F16" s="3" t="str">
+        <x:v>七号队（演示）</x:v>
+      </x:c>
+      <x:c r="G16" s="3" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="H16" s="3" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="I16" s="3" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="J16" s="3" t="str">
+        <x:v>优先录取</x:v>
+      </x:c>
+      <x:c r="K16" s="3" t="str">
+        <x:v>p-yeqing</x:v>
+      </x:c>
+      <x:c r="L16" s="3" t="str">
+        <x:v>叶青（演示）</x:v>
+      </x:c>
+      <x:c r="M16" s="10" t="n">
+        <x:v>46203.04166666667</x:v>
+      </x:c>
       <x:c r="N16" s="3" t="str">
         <x:v>xe-select-v1</x:v>
       </x:c>
       <x:c r="O16" s="3" t="str">
-        <x:v>缺段</x:v>
+        <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P16" s="3" t="str">
-        <x:v>演示重建：缺少入营选拔评审记录，未补造评价或评价人。</x:v>
+        <x:v>演示重建：组队作品，三人分工完成整套流程，演示由队长主讲；按同队各自一行记录。</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="48" customHeight="1">
@@ -1107,32 +1137,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D17" s="3" t="str">
-        <x:v>bow-923-work-016</x:v>
+        <x:v>bow-923-v3-work-016</x:v>
       </x:c>
       <x:c r="E17" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F17" s="3"/>
       <x:c r="G17" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H17" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I17" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J17" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="K17" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>p-yeqing</x:v>
       </x:c>
       <x:c r="L17" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>叶青（演示）</x:v>
       </x:c>
       <x:c r="M17" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N17" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -1141,7 +1171,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P17" s="3" t="str">
-        <x:v>演示重建：作品主流程完整，能说明一次方案取舍，并现场复现失败后的恢复步骤。</x:v>
+        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="48" customHeight="1">
@@ -1155,32 +1185,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D18" s="3" t="str">
-        <x:v>bow-923-work-017</x:v>
+        <x:v>bow-923-v3-work-017</x:v>
       </x:c>
       <x:c r="E18" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F18" s="3"/>
       <x:c r="G18" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H18" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="I18" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J18" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>刚过线</x:v>
       </x:c>
       <x:c r="K18" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>p-yeqing</x:v>
       </x:c>
       <x:c r="L18" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>叶青（演示）</x:v>
       </x:c>
       <x:c r="M18" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N18" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -1203,32 +1233,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D19" s="3" t="str">
-        <x:v>bow-923-work-018</x:v>
+        <x:v>bow-923-v3-work-018</x:v>
       </x:c>
       <x:c r="E19" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F19" s="3"/>
       <x:c r="G19" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H19" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I19" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J19" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>优先录取</x:v>
       </x:c>
       <x:c r="K19" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-28</x:v>
       </x:c>
       <x:c r="L19" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>许致远（演示）</x:v>
       </x:c>
       <x:c r="M19" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N19" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -1251,32 +1281,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D20" s="3" t="str">
-        <x:v>bow-923-work-019</x:v>
+        <x:v>bow-923-v3-work-019</x:v>
       </x:c>
       <x:c r="E20" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F20" s="3"/>
       <x:c r="G20" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H20" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="I20" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J20" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>刚过线</x:v>
       </x:c>
       <x:c r="K20" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-28</x:v>
       </x:c>
       <x:c r="L20" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>许致远（演示）</x:v>
       </x:c>
       <x:c r="M20" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N20" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -1285,7 +1315,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P20" s="3" t="str">
-        <x:v>演示重建：作品主流程完整，能说明一次方案取舍，并现场复现失败后的恢复步骤。</x:v>
+        <x:v>演示重建：完成了最小主流程；评审时未充分展示边界场景，按原档位记录。</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="48" customHeight="1">
@@ -1299,32 +1329,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D21" s="3" t="str">
-        <x:v>bow-923-work-020</x:v>
+        <x:v>bow-923-v3-work-020</x:v>
       </x:c>
       <x:c r="E21" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F21" s="3"/>
       <x:c r="G21" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H21" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I21" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J21" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>优先录取</x:v>
       </x:c>
       <x:c r="K21" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-28</x:v>
       </x:c>
       <x:c r="L21" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>许致远（演示）</x:v>
       </x:c>
       <x:c r="M21" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N21" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -1347,32 +1377,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D22" s="3" t="str">
-        <x:v>bow-923-work-021</x:v>
+        <x:v>bow-923-v3-work-021</x:v>
       </x:c>
       <x:c r="E22" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F22" s="3"/>
       <x:c r="G22" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H22" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I22" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J22" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>优先录取</x:v>
       </x:c>
       <x:c r="K22" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-28</x:v>
       </x:c>
       <x:c r="L22" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>许致远（演示）</x:v>
       </x:c>
       <x:c r="M22" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N22" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -1395,32 +1425,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D23" s="3" t="str">
-        <x:v>bow-923-work-022</x:v>
+        <x:v>bow-923-v3-work-022</x:v>
       </x:c>
       <x:c r="E23" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F23" s="3"/>
       <x:c r="G23" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H23" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I23" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J23" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>优先录取</x:v>
       </x:c>
       <x:c r="K23" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-28</x:v>
       </x:c>
       <x:c r="L23" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>许致远（演示）</x:v>
       </x:c>
       <x:c r="M23" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N23" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -1443,32 +1473,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D24" s="3" t="str">
-        <x:v>bow-923-work-023</x:v>
+        <x:v>bow-923-v3-work-023</x:v>
       </x:c>
       <x:c r="E24" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F24" s="3"/>
       <x:c r="G24" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H24" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I24" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J24" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="K24" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-28</x:v>
       </x:c>
       <x:c r="L24" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>许致远（演示）</x:v>
       </x:c>
       <x:c r="M24" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N24" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -1477,7 +1507,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P24" s="3" t="str">
-        <x:v>演示重建：作品主流程完整，能说明一次方案取舍，并现场复现失败后的恢复步骤。</x:v>
+        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="48" customHeight="1">
@@ -1491,32 +1521,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D25" s="3" t="str">
-        <x:v>bow-923-work-024</x:v>
+        <x:v>bow-923-v3-work-024</x:v>
       </x:c>
       <x:c r="E25" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F25" s="3"/>
       <x:c r="G25" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H25" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I25" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J25" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="K25" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-28</x:v>
       </x:c>
       <x:c r="L25" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>许致远（演示）</x:v>
       </x:c>
       <x:c r="M25" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N25" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -1525,7 +1555,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P25" s="3" t="str">
-        <x:v>演示重建：作品主流程完整，能说明一次方案取舍，并现场复现失败后的恢复步骤。</x:v>
+        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="48" customHeight="1">
@@ -1539,32 +1569,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D26" s="3" t="str">
-        <x:v>bow-923-work-025</x:v>
+        <x:v>bow-923-v3-work-025</x:v>
       </x:c>
       <x:c r="E26" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F26" s="3"/>
       <x:c r="G26" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H26" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I26" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J26" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="K26" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-28</x:v>
       </x:c>
       <x:c r="L26" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>许致远（演示）</x:v>
       </x:c>
       <x:c r="M26" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N26" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -1573,7 +1603,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P26" s="3" t="str">
-        <x:v>演示重建：作品主流程完整，能说明一次方案取舍，并现场复现失败后的恢复步骤。</x:v>
+        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="48" customHeight="1">
@@ -1587,32 +1617,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D27" s="3" t="str">
-        <x:v>bow-923-work-026</x:v>
+        <x:v>bow-923-v3-work-026</x:v>
       </x:c>
       <x:c r="E27" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F27" s="3"/>
       <x:c r="G27" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H27" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="I27" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J27" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>刚过线</x:v>
       </x:c>
       <x:c r="K27" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-28</x:v>
       </x:c>
       <x:c r="L27" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>许致远（演示）</x:v>
       </x:c>
       <x:c r="M27" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N27" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -1635,32 +1665,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D28" s="3" t="str">
-        <x:v>bow-923-work-027</x:v>
+        <x:v>bow-923-v3-work-027</x:v>
       </x:c>
       <x:c r="E28" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F28" s="3"/>
       <x:c r="G28" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H28" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I28" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J28" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>优先录取</x:v>
       </x:c>
       <x:c r="K28" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-28</x:v>
       </x:c>
       <x:c r="L28" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>许致远（演示）</x:v>
       </x:c>
       <x:c r="M28" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N28" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -1669,7 +1699,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P28" s="3" t="str">
-        <x:v>演示重建：完成了最小主流程；评审时未充分展示边界场景，按原档位记录。</x:v>
+        <x:v>演示重建：作品主流程完整，能说明一次方案取舍，并现场复现失败后的恢复步骤。</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="48" customHeight="1">
@@ -1683,32 +1713,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D29" s="3" t="str">
-        <x:v>bow-923-work-028</x:v>
+        <x:v>bow-923-v3-work-028</x:v>
       </x:c>
       <x:c r="E29" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F29" s="3"/>
       <x:c r="G29" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H29" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I29" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J29" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="K29" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-28</x:v>
       </x:c>
       <x:c r="L29" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>许致远（演示）</x:v>
       </x:c>
       <x:c r="M29" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N29" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -1717,7 +1747,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P29" s="3" t="str">
-        <x:v>演示重建：完成了最小主流程；评审时未充分展示边界场景，按原档位记录。</x:v>
+        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="48" customHeight="1">
@@ -1731,32 +1761,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D30" s="3" t="str">
-        <x:v>bow-923-work-029</x:v>
+        <x:v>bow-923-v3-work-029</x:v>
       </x:c>
       <x:c r="E30" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F30" s="3"/>
       <x:c r="G30" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H30" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I30" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J30" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>优先录取</x:v>
       </x:c>
       <x:c r="K30" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-28</x:v>
       </x:c>
       <x:c r="L30" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>许致远（演示）</x:v>
       </x:c>
       <x:c r="M30" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N30" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -1765,7 +1795,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P30" s="3" t="str">
-        <x:v>演示重建：完成了最小主流程；评审时未充分展示边界场景，按原档位记录。</x:v>
+        <x:v>演示重建：作品主流程完整，能说明一次方案取舍，并现场复现失败后的恢复步骤。</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="48" customHeight="1">
@@ -1779,32 +1809,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D31" s="3" t="str">
-        <x:v>bow-923-work-030</x:v>
+        <x:v>bow-923-v3-work-030</x:v>
       </x:c>
       <x:c r="E31" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F31" s="3"/>
       <x:c r="G31" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H31" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I31" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J31" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>优先录取</x:v>
       </x:c>
       <x:c r="K31" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-28</x:v>
       </x:c>
       <x:c r="L31" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>许致远（演示）</x:v>
       </x:c>
       <x:c r="M31" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N31" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -1813,7 +1843,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P31" s="3" t="str">
-        <x:v>演示重建：完成了最小主流程；评审时未充分展示边界场景，按原档位记录。</x:v>
+        <x:v>演示重建：作品主流程完整，能说明一次方案取舍，并现场复现失败后的恢复步骤。</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="48" customHeight="1">
@@ -1827,32 +1857,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D32" s="3" t="str">
-        <x:v>bow-923-work-031</x:v>
+        <x:v>bow-923-v3-work-031</x:v>
       </x:c>
       <x:c r="E32" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F32" s="3"/>
       <x:c r="G32" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H32" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I32" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J32" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="K32" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-28</x:v>
       </x:c>
       <x:c r="L32" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>许致远（演示）</x:v>
       </x:c>
       <x:c r="M32" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N32" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -1861,7 +1891,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P32" s="3" t="str">
-        <x:v>演示重建：完成了最小主流程；评审时未充分展示边界场景，按原档位记录。</x:v>
+        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="48" customHeight="1">
@@ -1875,32 +1905,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D33" s="3" t="str">
-        <x:v>bow-923-work-032</x:v>
+        <x:v>bow-923-v3-work-032</x:v>
       </x:c>
       <x:c r="E33" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F33" s="3"/>
       <x:c r="G33" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H33" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I33" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J33" s="3" t="str">
-        <x:v>刚过线档</x:v>
+        <x:v>优先录取</x:v>
       </x:c>
       <x:c r="K33" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-28</x:v>
       </x:c>
       <x:c r="L33" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>许致远（演示）</x:v>
       </x:c>
       <x:c r="M33" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N33" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -1909,7 +1939,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P33" s="3" t="str">
-        <x:v>演示重建：完成了最小主流程；评审时未充分展示边界场景，按原档位记录。</x:v>
+        <x:v>演示重建：作品主流程完整，能说明一次方案取舍，并现场复现失败后的恢复步骤。</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="48" customHeight="1">
@@ -1923,32 +1953,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D34" s="3" t="str">
-        <x:v>bow-923-work-033</x:v>
+        <x:v>bow-923-v3-work-033</x:v>
       </x:c>
       <x:c r="E34" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F34" s="3"/>
       <x:c r="G34" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H34" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I34" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J34" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>优先录取</x:v>
       </x:c>
       <x:c r="K34" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-28</x:v>
       </x:c>
       <x:c r="L34" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>许致远（演示）</x:v>
       </x:c>
       <x:c r="M34" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N34" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -1957,7 +1987,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P34" s="3" t="str">
-        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
+        <x:v>演示重建：作品主流程完整，能说明一次方案取舍，并现场复现失败后的恢复步骤。</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="48" customHeight="1">
@@ -1971,32 +2001,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D35" s="3" t="str">
-        <x:v>bow-923-work-034</x:v>
+        <x:v>bow-923-v3-work-034</x:v>
       </x:c>
       <x:c r="E35" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F35" s="3"/>
       <x:c r="G35" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H35" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I35" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J35" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="K35" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-28</x:v>
       </x:c>
       <x:c r="L35" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>许致远（演示）</x:v>
       </x:c>
       <x:c r="M35" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N35" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -2019,32 +2049,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D36" s="3" t="str">
-        <x:v>bow-923-work-035</x:v>
+        <x:v>bow-923-v3-work-035</x:v>
       </x:c>
       <x:c r="E36" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F36" s="3"/>
       <x:c r="G36" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H36" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="I36" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J36" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>刚过线</x:v>
       </x:c>
       <x:c r="K36" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-28</x:v>
       </x:c>
       <x:c r="L36" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>许致远（演示）</x:v>
       </x:c>
       <x:c r="M36" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N36" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -2053,7 +2083,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P36" s="3" t="str">
-        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
+        <x:v>演示重建：完成了最小主流程；评审时未充分展示边界场景，按原档位记录。</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="48" customHeight="1">
@@ -2067,32 +2097,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D37" s="3" t="str">
-        <x:v>bow-923-work-036</x:v>
+        <x:v>bow-923-v3-work-036</x:v>
       </x:c>
       <x:c r="E37" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F37" s="3"/>
       <x:c r="G37" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H37" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I37" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J37" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>优先录取</x:v>
       </x:c>
       <x:c r="K37" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-28</x:v>
       </x:c>
       <x:c r="L37" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>许致远（演示）</x:v>
       </x:c>
       <x:c r="M37" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N37" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -2101,7 +2131,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P37" s="3" t="str">
-        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
+        <x:v>演示重建：作品主流程完整，能说明一次方案取舍，并现场复现失败后的恢复步骤。</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="48" customHeight="1">
@@ -2115,32 +2145,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D38" s="3" t="str">
-        <x:v>bow-923-work-037</x:v>
+        <x:v>bow-923-v3-work-037</x:v>
       </x:c>
       <x:c r="E38" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F38" s="3"/>
       <x:c r="G38" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H38" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I38" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J38" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="K38" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-28</x:v>
       </x:c>
       <x:c r="L38" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>许致远（演示）</x:v>
       </x:c>
       <x:c r="M38" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N38" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -2163,32 +2193,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D39" s="3" t="str">
-        <x:v>bow-923-work-038</x:v>
+        <x:v>bow-923-v3-work-038</x:v>
       </x:c>
       <x:c r="E39" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F39" s="3"/>
       <x:c r="G39" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H39" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I39" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J39" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>优先录取</x:v>
       </x:c>
       <x:c r="K39" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-17</x:v>
       </x:c>
       <x:c r="L39" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>贺云舒（演示）</x:v>
       </x:c>
       <x:c r="M39" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N39" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -2197,7 +2227,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P39" s="3" t="str">
-        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
+        <x:v>演示重建：作品主流程完整，能说明一次方案取舍，并现场复现失败后的恢复步骤。</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="48" customHeight="1">
@@ -2211,32 +2241,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D40" s="3" t="str">
-        <x:v>bow-923-work-039</x:v>
+        <x:v>bow-923-v3-work-039</x:v>
       </x:c>
       <x:c r="E40" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F40" s="3"/>
       <x:c r="G40" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H40" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="I40" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J40" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>刚过线</x:v>
       </x:c>
       <x:c r="K40" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-17</x:v>
       </x:c>
       <x:c r="L40" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>贺云舒（演示）</x:v>
       </x:c>
       <x:c r="M40" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N40" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -2245,7 +2275,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P40" s="3" t="str">
-        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
+        <x:v>演示重建：完成了最小主流程；评审时未充分展示边界场景，按原档位记录。</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="48" customHeight="1">
@@ -2259,32 +2289,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D41" s="3" t="str">
-        <x:v>bow-923-work-040</x:v>
+        <x:v>bow-923-v3-work-040</x:v>
       </x:c>
       <x:c r="E41" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F41" s="3"/>
       <x:c r="G41" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H41" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I41" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J41" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="K41" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-17</x:v>
       </x:c>
       <x:c r="L41" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>贺云舒（演示）</x:v>
       </x:c>
       <x:c r="M41" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N41" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -2307,32 +2337,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D42" s="3" t="str">
-        <x:v>bow-923-work-041</x:v>
+        <x:v>bow-923-v3-work-041</x:v>
       </x:c>
       <x:c r="E42" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F42" s="3"/>
       <x:c r="G42" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H42" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="I42" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J42" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>刚过线</x:v>
       </x:c>
       <x:c r="K42" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-17</x:v>
       </x:c>
       <x:c r="L42" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>贺云舒（演示）</x:v>
       </x:c>
       <x:c r="M42" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N42" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -2341,7 +2371,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P42" s="3" t="str">
-        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
+        <x:v>演示重建：完成了最小主流程；评审时未充分展示边界场景，按原档位记录。</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="48" customHeight="1">
@@ -2355,32 +2385,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D43" s="3" t="str">
-        <x:v>bow-923-work-042</x:v>
+        <x:v>bow-923-v3-work-042</x:v>
       </x:c>
       <x:c r="E43" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F43" s="3"/>
       <x:c r="G43" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H43" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I43" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J43" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="K43" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-17</x:v>
       </x:c>
       <x:c r="L43" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>贺云舒（演示）</x:v>
       </x:c>
       <x:c r="M43" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N43" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -2403,32 +2433,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D44" s="3" t="str">
-        <x:v>bow-923-work-043</x:v>
+        <x:v>bow-923-v3-work-043</x:v>
       </x:c>
       <x:c r="E44" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F44" s="3"/>
       <x:c r="G44" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H44" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I44" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J44" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="K44" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-17</x:v>
       </x:c>
       <x:c r="L44" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>贺云舒（演示）</x:v>
       </x:c>
       <x:c r="M44" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N44" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -2451,32 +2481,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D45" s="3" t="str">
-        <x:v>bow-923-work-044</x:v>
+        <x:v>bow-923-v3-work-044</x:v>
       </x:c>
       <x:c r="E45" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F45" s="3"/>
       <x:c r="G45" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H45" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="I45" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J45" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>刚过线</x:v>
       </x:c>
       <x:c r="K45" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-17</x:v>
       </x:c>
       <x:c r="L45" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>贺云舒（演示）</x:v>
       </x:c>
       <x:c r="M45" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N45" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -2485,7 +2515,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P45" s="3" t="str">
-        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
+        <x:v>演示重建：完成了最小主流程；评审时未充分展示边界场景，按原档位记录。</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="48" customHeight="1">
@@ -2499,32 +2529,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D46" s="3" t="str">
-        <x:v>bow-923-work-045</x:v>
+        <x:v>bow-923-v3-work-045</x:v>
       </x:c>
       <x:c r="E46" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F46" s="3"/>
       <x:c r="G46" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H46" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="I46" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J46" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>刚过线</x:v>
       </x:c>
       <x:c r="K46" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-17</x:v>
       </x:c>
       <x:c r="L46" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>贺云舒（演示）</x:v>
       </x:c>
       <x:c r="M46" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N46" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -2533,7 +2563,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P46" s="3" t="str">
-        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
+        <x:v>演示重建：完成了最小主流程；评审时未充分展示边界场景，按原档位记录。</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="48" customHeight="1">
@@ -2547,32 +2577,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D47" s="3" t="str">
-        <x:v>bow-923-work-046</x:v>
+        <x:v>bow-923-v3-work-046</x:v>
       </x:c>
       <x:c r="E47" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F47" s="3"/>
       <x:c r="G47" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H47" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I47" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J47" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="K47" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-17</x:v>
       </x:c>
       <x:c r="L47" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>贺云舒（演示）</x:v>
       </x:c>
       <x:c r="M47" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N47" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -2595,41 +2625,27 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D48" s="3" t="str">
-        <x:v>bow-923-work-047</x:v>
+        <x:v>bow-923-v3-work-047</x:v>
       </x:c>
       <x:c r="E48" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F48" s="3"/>
-      <x:c r="G48" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="H48" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="I48" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="J48" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="K48" s="3" t="str">
-        <x:v>s-04</x:v>
-      </x:c>
-      <x:c r="L48" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
-      </x:c>
-      <x:c r="M48" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
-      </x:c>
+      <x:c r="G48" s="3"/>
+      <x:c r="H48" s="3"/>
+      <x:c r="I48" s="3"/>
+      <x:c r="J48" s="3"/>
+      <x:c r="K48" s="3"/>
+      <x:c r="L48" s="3"/>
+      <x:c r="M48" s="10"/>
       <x:c r="N48" s="3" t="str">
         <x:v>xe-select-v1</x:v>
       </x:c>
       <x:c r="O48" s="3" t="str">
-        <x:v>已确认（演示）</x:v>
+        <x:v>缺段</x:v>
       </x:c>
       <x:c r="P48" s="3" t="str">
-        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
+        <x:v>演示重建：第二批次补录入营，没有参加作品评审，未补造评价或评价人。</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="48" customHeight="1">
@@ -2643,41 +2659,27 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D49" s="3" t="str">
-        <x:v>bow-923-work-048</x:v>
+        <x:v>bow-923-v3-work-048</x:v>
       </x:c>
       <x:c r="E49" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F49" s="3"/>
-      <x:c r="G49" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="H49" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="I49" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="J49" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="K49" s="3" t="str">
-        <x:v>s-04</x:v>
-      </x:c>
-      <x:c r="L49" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
-      </x:c>
-      <x:c r="M49" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
-      </x:c>
+      <x:c r="G49" s="3"/>
+      <x:c r="H49" s="3"/>
+      <x:c r="I49" s="3"/>
+      <x:c r="J49" s="3"/>
+      <x:c r="K49" s="3"/>
+      <x:c r="L49" s="3"/>
+      <x:c r="M49" s="10"/>
       <x:c r="N49" s="3" t="str">
         <x:v>xe-select-v1</x:v>
       </x:c>
       <x:c r="O49" s="3" t="str">
-        <x:v>已确认（演示）</x:v>
+        <x:v>缺段</x:v>
       </x:c>
       <x:c r="P49" s="3" t="str">
-        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
+        <x:v>演示重建：第二批次补录入营，没有参加作品评审，未补造评价或评价人。</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="48" customHeight="1">
@@ -2691,41 +2693,27 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D50" s="3" t="str">
-        <x:v>bow-923-work-049</x:v>
+        <x:v>bow-923-v3-work-049</x:v>
       </x:c>
       <x:c r="E50" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F50" s="3"/>
-      <x:c r="G50" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="H50" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="I50" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="J50" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="K50" s="3" t="str">
-        <x:v>s-04</x:v>
-      </x:c>
-      <x:c r="L50" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
-      </x:c>
-      <x:c r="M50" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
-      </x:c>
+      <x:c r="G50" s="3"/>
+      <x:c r="H50" s="3"/>
+      <x:c r="I50" s="3"/>
+      <x:c r="J50" s="3"/>
+      <x:c r="K50" s="3"/>
+      <x:c r="L50" s="3"/>
+      <x:c r="M50" s="10"/>
       <x:c r="N50" s="3" t="str">
         <x:v>xe-select-v1</x:v>
       </x:c>
       <x:c r="O50" s="3" t="str">
-        <x:v>已确认（演示）</x:v>
+        <x:v>缺段</x:v>
       </x:c>
       <x:c r="P50" s="3" t="str">
-        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
+        <x:v>演示重建：第二批次补录入营，没有参加作品评审，未补造评价或评价人。</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="48" customHeight="1">
@@ -2739,41 +2727,27 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D51" s="3" t="str">
-        <x:v>bow-923-work-050</x:v>
+        <x:v>bow-923-v3-work-050</x:v>
       </x:c>
       <x:c r="E51" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F51" s="3"/>
-      <x:c r="G51" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="H51" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="I51" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="J51" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="K51" s="3" t="str">
-        <x:v>s-04</x:v>
-      </x:c>
-      <x:c r="L51" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
-      </x:c>
-      <x:c r="M51" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
-      </x:c>
+      <x:c r="G51" s="3"/>
+      <x:c r="H51" s="3"/>
+      <x:c r="I51" s="3"/>
+      <x:c r="J51" s="3"/>
+      <x:c r="K51" s="3"/>
+      <x:c r="L51" s="3"/>
+      <x:c r="M51" s="10"/>
       <x:c r="N51" s="3" t="str">
         <x:v>xe-select-v1</x:v>
       </x:c>
       <x:c r="O51" s="3" t="str">
-        <x:v>已确认（演示）</x:v>
+        <x:v>缺段</x:v>
       </x:c>
       <x:c r="P51" s="3" t="str">
-        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
+        <x:v>演示重建：第二批次补录入营，没有参加作品评审，未补造评价或评价人。</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="48" customHeight="1">
@@ -2787,41 +2761,27 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D52" s="3" t="str">
-        <x:v>bow-923-work-051</x:v>
+        <x:v>bow-923-v3-work-051</x:v>
       </x:c>
       <x:c r="E52" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F52" s="3"/>
-      <x:c r="G52" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="H52" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="I52" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="J52" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="K52" s="3" t="str">
-        <x:v>s-04</x:v>
-      </x:c>
-      <x:c r="L52" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
-      </x:c>
-      <x:c r="M52" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
-      </x:c>
+      <x:c r="G52" s="3"/>
+      <x:c r="H52" s="3"/>
+      <x:c r="I52" s="3"/>
+      <x:c r="J52" s="3"/>
+      <x:c r="K52" s="3"/>
+      <x:c r="L52" s="3"/>
+      <x:c r="M52" s="10"/>
       <x:c r="N52" s="3" t="str">
         <x:v>xe-select-v1</x:v>
       </x:c>
       <x:c r="O52" s="3" t="str">
-        <x:v>已确认（演示）</x:v>
+        <x:v>缺段</x:v>
       </x:c>
       <x:c r="P52" s="3" t="str">
-        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
+        <x:v>演示重建：第二批次补录入营，没有参加作品评审，未补造评价或评价人。</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="48" customHeight="1">
@@ -2835,41 +2795,27 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D53" s="3" t="str">
-        <x:v>bow-923-work-052</x:v>
+        <x:v>bow-923-v3-work-052</x:v>
       </x:c>
       <x:c r="E53" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F53" s="3"/>
-      <x:c r="G53" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="H53" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="I53" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="J53" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="K53" s="3" t="str">
-        <x:v>s-04</x:v>
-      </x:c>
-      <x:c r="L53" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
-      </x:c>
-      <x:c r="M53" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
-      </x:c>
+      <x:c r="G53" s="3"/>
+      <x:c r="H53" s="3"/>
+      <x:c r="I53" s="3"/>
+      <x:c r="J53" s="3"/>
+      <x:c r="K53" s="3"/>
+      <x:c r="L53" s="3"/>
+      <x:c r="M53" s="10"/>
       <x:c r="N53" s="3" t="str">
         <x:v>xe-select-v1</x:v>
       </x:c>
       <x:c r="O53" s="3" t="str">
-        <x:v>已确认（演示）</x:v>
+        <x:v>缺段</x:v>
       </x:c>
       <x:c r="P53" s="3" t="str">
-        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
+        <x:v>演示重建：第二批次补录入营，没有参加作品评审，未补造评价或评价人。</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="48" customHeight="1">
@@ -2883,41 +2829,27 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D54" s="3" t="str">
-        <x:v>bow-923-work-053</x:v>
+        <x:v>bow-923-v3-work-053</x:v>
       </x:c>
       <x:c r="E54" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F54" s="3"/>
-      <x:c r="G54" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="H54" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="I54" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="J54" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="K54" s="3" t="str">
-        <x:v>s-04</x:v>
-      </x:c>
-      <x:c r="L54" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
-      </x:c>
-      <x:c r="M54" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
-      </x:c>
+      <x:c r="G54" s="3"/>
+      <x:c r="H54" s="3"/>
+      <x:c r="I54" s="3"/>
+      <x:c r="J54" s="3"/>
+      <x:c r="K54" s="3"/>
+      <x:c r="L54" s="3"/>
+      <x:c r="M54" s="10"/>
       <x:c r="N54" s="3" t="str">
         <x:v>xe-select-v1</x:v>
       </x:c>
       <x:c r="O54" s="3" t="str">
-        <x:v>已确认（演示）</x:v>
+        <x:v>缺段</x:v>
       </x:c>
       <x:c r="P54" s="3" t="str">
-        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
+        <x:v>演示重建：第二批次补录入营，没有参加作品评审，未补造评价或评价人。</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="48" customHeight="1">
@@ -2931,41 +2863,27 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D55" s="3" t="str">
-        <x:v>bow-923-work-054</x:v>
+        <x:v>bow-923-v3-work-054</x:v>
       </x:c>
       <x:c r="E55" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F55" s="3"/>
-      <x:c r="G55" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="H55" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="I55" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="J55" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="K55" s="3" t="str">
-        <x:v>s-04</x:v>
-      </x:c>
-      <x:c r="L55" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
-      </x:c>
-      <x:c r="M55" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
-      </x:c>
+      <x:c r="G55" s="3"/>
+      <x:c r="H55" s="3"/>
+      <x:c r="I55" s="3"/>
+      <x:c r="J55" s="3"/>
+      <x:c r="K55" s="3"/>
+      <x:c r="L55" s="3"/>
+      <x:c r="M55" s="10"/>
       <x:c r="N55" s="3" t="str">
         <x:v>xe-select-v1</x:v>
       </x:c>
       <x:c r="O55" s="3" t="str">
-        <x:v>已确认（演示）</x:v>
+        <x:v>缺段</x:v>
       </x:c>
       <x:c r="P55" s="3" t="str">
-        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
+        <x:v>演示重建：第二批次补录入营，没有参加作品评审，未补造评价或评价人。</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="48" customHeight="1">
@@ -2979,41 +2897,27 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D56" s="3" t="str">
-        <x:v>bow-923-work-055</x:v>
+        <x:v>bow-923-v3-work-055</x:v>
       </x:c>
       <x:c r="E56" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F56" s="3"/>
-      <x:c r="G56" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="H56" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="I56" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="J56" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="K56" s="3" t="str">
-        <x:v>s-04</x:v>
-      </x:c>
-      <x:c r="L56" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
-      </x:c>
-      <x:c r="M56" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
-      </x:c>
+      <x:c r="G56" s="3"/>
+      <x:c r="H56" s="3"/>
+      <x:c r="I56" s="3"/>
+      <x:c r="J56" s="3"/>
+      <x:c r="K56" s="3"/>
+      <x:c r="L56" s="3"/>
+      <x:c r="M56" s="10"/>
       <x:c r="N56" s="3" t="str">
         <x:v>xe-select-v1</x:v>
       </x:c>
       <x:c r="O56" s="3" t="str">
-        <x:v>已确认（演示）</x:v>
+        <x:v>缺段</x:v>
       </x:c>
       <x:c r="P56" s="3" t="str">
-        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
+        <x:v>演示重建：第二批次补录入营，没有参加作品评审，未补造评价或评价人。</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="48" customHeight="1">
@@ -3027,41 +2931,27 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D57" s="3" t="str">
-        <x:v>bow-923-work-056</x:v>
+        <x:v>bow-923-v3-work-056</x:v>
       </x:c>
       <x:c r="E57" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F57" s="3"/>
-      <x:c r="G57" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="H57" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="I57" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="J57" s="3" t="str">
-        <x:v>中间档</x:v>
-      </x:c>
-      <x:c r="K57" s="3" t="str">
-        <x:v>s-04</x:v>
-      </x:c>
-      <x:c r="L57" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
-      </x:c>
-      <x:c r="M57" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
-      </x:c>
+      <x:c r="G57" s="3"/>
+      <x:c r="H57" s="3"/>
+      <x:c r="I57" s="3"/>
+      <x:c r="J57" s="3"/>
+      <x:c r="K57" s="3"/>
+      <x:c r="L57" s="3"/>
+      <x:c r="M57" s="10"/>
       <x:c r="N57" s="3" t="str">
         <x:v>xe-select-v1</x:v>
       </x:c>
       <x:c r="O57" s="3" t="str">
-        <x:v>已确认（演示）</x:v>
+        <x:v>缺段</x:v>
       </x:c>
       <x:c r="P57" s="3" t="str">
-        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
+        <x:v>演示重建：第二批次补录入营，没有参加作品评审，未补造评价或评价人。</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="48" customHeight="1">
@@ -3075,32 +2965,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D58" s="3" t="str">
-        <x:v>bow-923-work-057</x:v>
+        <x:v>bow-923-v3-work-057</x:v>
       </x:c>
       <x:c r="E58" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F58" s="3"/>
       <x:c r="G58" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H58" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="I58" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J58" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>刚过线</x:v>
       </x:c>
       <x:c r="K58" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-28</x:v>
       </x:c>
       <x:c r="L58" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>许致远（演示）</x:v>
       </x:c>
       <x:c r="M58" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N58" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -3109,7 +2999,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P58" s="3" t="str">
-        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
+        <x:v>演示重建：完成了最小主流程；评审时未充分展示边界场景，按原档位记录。</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="48" customHeight="1">
@@ -3123,32 +3013,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D59" s="3" t="str">
-        <x:v>bow-923-work-058</x:v>
+        <x:v>bow-923-v3-work-058</x:v>
       </x:c>
       <x:c r="E59" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F59" s="3"/>
       <x:c r="G59" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H59" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="I59" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J59" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>刚过线</x:v>
       </x:c>
       <x:c r="K59" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>p-yeqing</x:v>
       </x:c>
       <x:c r="L59" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>叶青（演示）</x:v>
       </x:c>
       <x:c r="M59" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N59" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -3157,7 +3047,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P59" s="3" t="str">
-        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
+        <x:v>演示重建：完成了最小主流程；评审时未充分展示边界场景，按原档位记录。</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="48" customHeight="1">
@@ -3171,32 +3061,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D60" s="3" t="str">
-        <x:v>bow-923-work-059</x:v>
+        <x:v>bow-923-v3-work-059</x:v>
       </x:c>
       <x:c r="E60" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F60" s="3"/>
       <x:c r="G60" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H60" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I60" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J60" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="K60" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-28</x:v>
       </x:c>
       <x:c r="L60" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>许致远（演示）</x:v>
       </x:c>
       <x:c r="M60" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N60" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -3219,32 +3109,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D61" s="3" t="str">
-        <x:v>bow-923-work-060</x:v>
+        <x:v>bow-923-v3-work-060</x:v>
       </x:c>
       <x:c r="E61" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F61" s="3"/>
       <x:c r="G61" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H61" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I61" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J61" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="K61" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-28</x:v>
       </x:c>
       <x:c r="L61" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>许致远（演示）</x:v>
       </x:c>
       <x:c r="M61" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N61" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -3267,32 +3157,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D62" s="3" t="str">
-        <x:v>bow-923-work-061</x:v>
+        <x:v>bow-923-v3-work-061</x:v>
       </x:c>
       <x:c r="E62" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F62" s="3"/>
       <x:c r="G62" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H62" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I62" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J62" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>优先录取</x:v>
       </x:c>
       <x:c r="K62" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-28</x:v>
       </x:c>
       <x:c r="L62" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>许致远（演示）</x:v>
       </x:c>
       <x:c r="M62" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N62" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -3301,7 +3191,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P62" s="3" t="str">
-        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
+        <x:v>演示重建：作品主流程完整，能说明一次方案取舍，并现场复现失败后的恢复步骤。</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="48" customHeight="1">
@@ -3315,32 +3205,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D63" s="3" t="str">
-        <x:v>bow-923-work-062</x:v>
+        <x:v>bow-923-v3-work-062</x:v>
       </x:c>
       <x:c r="E63" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F63" s="3"/>
       <x:c r="G63" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H63" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I63" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J63" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="K63" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-28</x:v>
       </x:c>
       <x:c r="L63" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>许致远（演示）</x:v>
       </x:c>
       <x:c r="M63" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N63" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -3363,32 +3253,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D64" s="3" t="str">
-        <x:v>bow-923-work-063</x:v>
+        <x:v>bow-923-v3-work-063</x:v>
       </x:c>
       <x:c r="E64" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F64" s="3"/>
       <x:c r="G64" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H64" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I64" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J64" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>优先录取</x:v>
       </x:c>
       <x:c r="K64" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-28</x:v>
       </x:c>
       <x:c r="L64" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>许致远（演示）</x:v>
       </x:c>
       <x:c r="M64" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N64" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -3397,7 +3287,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P64" s="3" t="str">
-        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
+        <x:v>演示重建：作品主流程完整，能说明一次方案取舍，并现场复现失败后的恢复步骤。</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="48" customHeight="1">
@@ -3411,32 +3301,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D65" s="3" t="str">
-        <x:v>bow-923-work-064</x:v>
+        <x:v>bow-923-v3-work-064</x:v>
       </x:c>
       <x:c r="E65" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F65" s="3"/>
       <x:c r="G65" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H65" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I65" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J65" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="K65" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-28</x:v>
       </x:c>
       <x:c r="L65" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>许致远（演示）</x:v>
       </x:c>
       <x:c r="M65" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N65" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -3459,32 +3349,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D66" s="3" t="str">
-        <x:v>bow-923-work-065</x:v>
+        <x:v>bow-923-v3-work-065</x:v>
       </x:c>
       <x:c r="E66" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F66" s="3"/>
       <x:c r="G66" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H66" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I66" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J66" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="K66" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-28</x:v>
       </x:c>
       <x:c r="L66" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>许致远（演示）</x:v>
       </x:c>
       <x:c r="M66" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N66" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -3507,32 +3397,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D67" s="3" t="str">
-        <x:v>bow-923-work-066</x:v>
+        <x:v>bow-923-v3-work-066</x:v>
       </x:c>
       <x:c r="E67" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F67" s="3"/>
       <x:c r="G67" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H67" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I67" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J67" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>优先录取</x:v>
       </x:c>
       <x:c r="K67" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-28</x:v>
       </x:c>
       <x:c r="L67" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>许致远（演示）</x:v>
       </x:c>
       <x:c r="M67" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N67" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -3541,7 +3431,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P67" s="3" t="str">
-        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
+        <x:v>演示重建：作品主流程完整，能说明一次方案取舍，并现场复现失败后的恢复步骤。</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="48" customHeight="1">
@@ -3555,32 +3445,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D68" s="3" t="str">
-        <x:v>bow-923-work-067</x:v>
+        <x:v>bow-923-v3-work-067</x:v>
       </x:c>
       <x:c r="E68" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F68" s="3"/>
       <x:c r="G68" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H68" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I68" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J68" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>优先录取</x:v>
       </x:c>
       <x:c r="K68" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-17</x:v>
       </x:c>
       <x:c r="L68" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>贺云舒（演示）</x:v>
       </x:c>
       <x:c r="M68" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N68" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -3589,7 +3479,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P68" s="3" t="str">
-        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
+        <x:v>演示重建：作品主流程完整，能说明一次方案取舍，并现场复现失败后的恢复步骤。</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="48" customHeight="1">
@@ -3603,32 +3493,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D69" s="3" t="str">
-        <x:v>bow-923-work-068</x:v>
+        <x:v>bow-923-v3-work-068</x:v>
       </x:c>
       <x:c r="E69" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F69" s="3"/>
       <x:c r="G69" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H69" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I69" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J69" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="K69" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-17</x:v>
       </x:c>
       <x:c r="L69" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>贺云舒（演示）</x:v>
       </x:c>
       <x:c r="M69" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N69" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -3651,32 +3541,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D70" s="3" t="str">
-        <x:v>bow-923-work-069</x:v>
+        <x:v>bow-923-v3-work-069</x:v>
       </x:c>
       <x:c r="E70" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F70" s="3"/>
       <x:c r="G70" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H70" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I70" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J70" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="K70" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-17</x:v>
       </x:c>
       <x:c r="L70" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>贺云舒（演示）</x:v>
       </x:c>
       <x:c r="M70" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N70" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -3699,32 +3589,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D71" s="3" t="str">
-        <x:v>bow-923-work-070</x:v>
+        <x:v>bow-923-v3-work-070</x:v>
       </x:c>
       <x:c r="E71" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F71" s="3"/>
       <x:c r="G71" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H71" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I71" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J71" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>优先录取</x:v>
       </x:c>
       <x:c r="K71" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-17</x:v>
       </x:c>
       <x:c r="L71" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>贺云舒（演示）</x:v>
       </x:c>
       <x:c r="M71" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N71" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -3733,7 +3623,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P71" s="3" t="str">
-        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
+        <x:v>演示重建：作品主流程完整，能说明一次方案取舍，并现场复现失败后的恢复步骤。</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="48" customHeight="1">
@@ -3747,32 +3637,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D72" s="3" t="str">
-        <x:v>bow-923-work-071</x:v>
+        <x:v>bow-923-v3-work-071</x:v>
       </x:c>
       <x:c r="E72" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F72" s="3"/>
       <x:c r="G72" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H72" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I72" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J72" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="K72" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-17</x:v>
       </x:c>
       <x:c r="L72" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>贺云舒（演示）</x:v>
       </x:c>
       <x:c r="M72" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N72" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -3795,32 +3685,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D73" s="3" t="str">
-        <x:v>bow-923-work-072</x:v>
+        <x:v>bow-923-v3-work-072</x:v>
       </x:c>
       <x:c r="E73" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F73" s="3"/>
       <x:c r="G73" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H73" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I73" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J73" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>优先录取</x:v>
       </x:c>
       <x:c r="K73" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-17</x:v>
       </x:c>
       <x:c r="L73" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>贺云舒（演示）</x:v>
       </x:c>
       <x:c r="M73" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N73" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -3829,7 +3719,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P73" s="3" t="str">
-        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
+        <x:v>演示重建：作品主流程完整，能说明一次方案取舍，并现场复现失败后的恢复步骤。</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="48" customHeight="1">
@@ -3843,32 +3733,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D74" s="3" t="str">
-        <x:v>bow-923-work-073</x:v>
+        <x:v>bow-923-v3-work-073</x:v>
       </x:c>
       <x:c r="E74" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F74" s="3"/>
       <x:c r="G74" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H74" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="I74" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J74" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>刚过线</x:v>
       </x:c>
       <x:c r="K74" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-17</x:v>
       </x:c>
       <x:c r="L74" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>贺云舒（演示）</x:v>
       </x:c>
       <x:c r="M74" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N74" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -3877,7 +3767,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P74" s="3" t="str">
-        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
+        <x:v>演示重建：完成了最小主流程；评审时未充分展示边界场景，按原档位记录。</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="48" customHeight="1">
@@ -3891,32 +3781,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D75" s="3" t="str">
-        <x:v>bow-923-work-074</x:v>
+        <x:v>bow-923-v3-work-074</x:v>
       </x:c>
       <x:c r="E75" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F75" s="3"/>
       <x:c r="G75" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H75" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="I75" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J75" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>刚过线</x:v>
       </x:c>
       <x:c r="K75" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-17</x:v>
       </x:c>
       <x:c r="L75" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>贺云舒（演示）</x:v>
       </x:c>
       <x:c r="M75" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N75" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -3925,7 +3815,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P75" s="3" t="str">
-        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
+        <x:v>演示重建：完成了最小主流程；评审时未充分展示边界场景，按原档位记录。</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="48" customHeight="1">
@@ -3939,32 +3829,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D76" s="3" t="str">
-        <x:v>bow-923-work-075</x:v>
+        <x:v>bow-923-v3-work-075</x:v>
       </x:c>
       <x:c r="E76" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F76" s="3"/>
       <x:c r="G76" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H76" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I76" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J76" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>优先录取</x:v>
       </x:c>
       <x:c r="K76" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-17</x:v>
       </x:c>
       <x:c r="L76" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>贺云舒（演示）</x:v>
       </x:c>
       <x:c r="M76" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N76" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -3973,7 +3863,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P76" s="3" t="str">
-        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
+        <x:v>演示重建：作品主流程完整，能说明一次方案取舍，并现场复现失败后的恢复步骤。</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="48" customHeight="1">
@@ -3987,32 +3877,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D77" s="3" t="str">
-        <x:v>bow-923-work-076</x:v>
+        <x:v>bow-923-v3-work-076</x:v>
       </x:c>
       <x:c r="E77" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F77" s="3"/>
       <x:c r="G77" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H77" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="I77" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J77" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>刚过线</x:v>
       </x:c>
       <x:c r="K77" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-17</x:v>
       </x:c>
       <x:c r="L77" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>贺云舒（演示）</x:v>
       </x:c>
       <x:c r="M77" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N77" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -4021,7 +3911,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P77" s="3" t="str">
-        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
+        <x:v>演示重建：完成了最小主流程；评审时未充分展示边界场景，按原档位记录。</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="48" customHeight="1">
@@ -4035,32 +3925,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D78" s="3" t="str">
-        <x:v>bow-923-work-077</x:v>
+        <x:v>bow-923-v3-work-077</x:v>
       </x:c>
       <x:c r="E78" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F78" s="3"/>
       <x:c r="G78" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H78" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I78" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J78" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="K78" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-17</x:v>
       </x:c>
       <x:c r="L78" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>贺云舒（演示）</x:v>
       </x:c>
       <x:c r="M78" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N78" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -4083,32 +3973,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D79" s="3" t="str">
-        <x:v>bow-923-work-078</x:v>
+        <x:v>bow-923-v3-work-078</x:v>
       </x:c>
       <x:c r="E79" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F79" s="3"/>
       <x:c r="G79" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H79" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="I79" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J79" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>刚过线</x:v>
       </x:c>
       <x:c r="K79" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-17</x:v>
       </x:c>
       <x:c r="L79" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>贺云舒（演示）</x:v>
       </x:c>
       <x:c r="M79" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N79" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -4117,7 +4007,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P79" s="3" t="str">
-        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
+        <x:v>演示重建：完成了最小主流程；评审时未充分展示边界场景，按原档位记录。</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="48" customHeight="1">
@@ -4131,32 +4021,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D80" s="3" t="str">
-        <x:v>bow-923-work-079</x:v>
+        <x:v>bow-923-v3-work-079</x:v>
       </x:c>
       <x:c r="E80" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F80" s="3"/>
       <x:c r="G80" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H80" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I80" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J80" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="K80" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-17</x:v>
       </x:c>
       <x:c r="L80" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>贺云舒（演示）</x:v>
       </x:c>
       <x:c r="M80" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N80" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -4179,32 +4069,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D81" s="3" t="str">
-        <x:v>bow-923-work-080</x:v>
+        <x:v>bow-923-v3-work-080</x:v>
       </x:c>
       <x:c r="E81" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F81" s="3"/>
       <x:c r="G81" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H81" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I81" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J81" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="K81" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-17</x:v>
       </x:c>
       <x:c r="L81" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>贺云舒（演示）</x:v>
       </x:c>
       <x:c r="M81" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N81" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -4227,32 +4117,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D82" s="3" t="str">
-        <x:v>bow-923-work-081</x:v>
+        <x:v>bow-923-v3-work-081</x:v>
       </x:c>
       <x:c r="E82" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F82" s="3"/>
       <x:c r="G82" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H82" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="I82" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J82" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>刚过线</x:v>
       </x:c>
       <x:c r="K82" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-17</x:v>
       </x:c>
       <x:c r="L82" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>贺云舒（演示）</x:v>
       </x:c>
       <x:c r="M82" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N82" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -4261,7 +4151,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P82" s="3" t="str">
-        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
+        <x:v>演示重建：完成了最小主流程；评审时未充分展示边界场景，按原档位记录。</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="48" customHeight="1">
@@ -4275,32 +4165,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D83" s="3" t="str">
-        <x:v>bow-923-work-082</x:v>
+        <x:v>bow-923-v3-work-082</x:v>
       </x:c>
       <x:c r="E83" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F83" s="3"/>
       <x:c r="G83" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H83" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I83" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J83" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>优先录取</x:v>
       </x:c>
       <x:c r="K83" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-12</x:v>
       </x:c>
       <x:c r="L83" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>谷牧野（演示）</x:v>
       </x:c>
       <x:c r="M83" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N83" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -4309,7 +4199,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P83" s="3" t="str">
-        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
+        <x:v>演示重建：作品主流程完整，能说明一次方案取舍，并现场复现失败后的恢复步骤。</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="48" customHeight="1">
@@ -4323,32 +4213,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D84" s="3" t="str">
-        <x:v>bow-923-work-083</x:v>
+        <x:v>bow-923-v3-work-083</x:v>
       </x:c>
       <x:c r="E84" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F84" s="3"/>
       <x:c r="G84" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H84" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I84" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J84" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="K84" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-12</x:v>
       </x:c>
       <x:c r="L84" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>谷牧野（演示）</x:v>
       </x:c>
       <x:c r="M84" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N84" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -4371,32 +4261,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D85" s="3" t="str">
-        <x:v>bow-923-work-084</x:v>
+        <x:v>bow-923-v3-work-084</x:v>
       </x:c>
       <x:c r="E85" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F85" s="3"/>
       <x:c r="G85" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H85" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="I85" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J85" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>刚过线</x:v>
       </x:c>
       <x:c r="K85" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-12</x:v>
       </x:c>
       <x:c r="L85" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>谷牧野（演示）</x:v>
       </x:c>
       <x:c r="M85" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N85" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -4405,7 +4295,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P85" s="3" t="str">
-        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
+        <x:v>演示重建：完成了最小主流程；评审时未充分展示边界场景，按原档位记录。</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="48" customHeight="1">
@@ -4419,27 +4309,41 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D86" s="3" t="str">
-        <x:v>bow-923-work-085</x:v>
+        <x:v>bow-923-v3-work-085</x:v>
       </x:c>
       <x:c r="E86" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F86" s="3"/>
-      <x:c r="G86" s="3"/>
-      <x:c r="H86" s="3"/>
-      <x:c r="I86" s="3"/>
-      <x:c r="J86" s="3"/>
-      <x:c r="K86" s="3"/>
-      <x:c r="L86" s="3"/>
-      <x:c r="M86" s="10"/>
+      <x:c r="G86" s="3" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="H86" s="3" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="I86" s="3" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="J86" s="3" t="str">
+        <x:v>优先录取</x:v>
+      </x:c>
+      <x:c r="K86" s="3" t="str">
+        <x:v>s-12</x:v>
+      </x:c>
+      <x:c r="L86" s="3" t="str">
+        <x:v>谷牧野（演示）</x:v>
+      </x:c>
+      <x:c r="M86" s="10" t="n">
+        <x:v>46203.04166666667</x:v>
+      </x:c>
       <x:c r="N86" s="3" t="str">
         <x:v>xe-select-v1</x:v>
       </x:c>
       <x:c r="O86" s="3" t="str">
-        <x:v>缺段</x:v>
+        <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P86" s="3" t="str">
-        <x:v>演示重建：缺少入营选拔评审记录，未补造评价或评价人。</x:v>
+        <x:v>演示重建：作品主流程完整，能说明一次方案取舍，并现场复现失败后的恢复步骤。</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="48" customHeight="1">
@@ -4453,27 +4357,41 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D87" s="3" t="str">
-        <x:v>bow-923-work-086</x:v>
+        <x:v>bow-923-v3-work-086</x:v>
       </x:c>
       <x:c r="E87" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F87" s="3"/>
-      <x:c r="G87" s="3"/>
-      <x:c r="H87" s="3"/>
-      <x:c r="I87" s="3"/>
-      <x:c r="J87" s="3"/>
-      <x:c r="K87" s="3"/>
-      <x:c r="L87" s="3"/>
-      <x:c r="M87" s="10"/>
+      <x:c r="G87" s="3" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="H87" s="3" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="I87" s="3" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="J87" s="3" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="K87" s="3" t="str">
+        <x:v>s-17</x:v>
+      </x:c>
+      <x:c r="L87" s="3" t="str">
+        <x:v>贺云舒（演示）</x:v>
+      </x:c>
+      <x:c r="M87" s="10" t="n">
+        <x:v>46203.04166666667</x:v>
+      </x:c>
       <x:c r="N87" s="3" t="str">
         <x:v>xe-select-v1</x:v>
       </x:c>
       <x:c r="O87" s="3" t="str">
-        <x:v>缺段</x:v>
+        <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P87" s="3" t="str">
-        <x:v>演示重建：缺少入营选拔评审记录，未补造评价或评价人。</x:v>
+        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="48" customHeight="1">
@@ -4487,27 +4405,41 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D88" s="3" t="str">
-        <x:v>bow-923-work-087</x:v>
+        <x:v>bow-923-v3-work-087</x:v>
       </x:c>
       <x:c r="E88" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F88" s="3"/>
-      <x:c r="G88" s="3"/>
-      <x:c r="H88" s="3"/>
-      <x:c r="I88" s="3"/>
-      <x:c r="J88" s="3"/>
-      <x:c r="K88" s="3"/>
-      <x:c r="L88" s="3"/>
-      <x:c r="M88" s="10"/>
+      <x:c r="G88" s="3" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="H88" s="3" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I88" s="3" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="J88" s="3" t="str">
+        <x:v>刚过线</x:v>
+      </x:c>
+      <x:c r="K88" s="3" t="str">
+        <x:v>s-17</x:v>
+      </x:c>
+      <x:c r="L88" s="3" t="str">
+        <x:v>贺云舒（演示）</x:v>
+      </x:c>
+      <x:c r="M88" s="10" t="n">
+        <x:v>46203.04166666667</x:v>
+      </x:c>
       <x:c r="N88" s="3" t="str">
         <x:v>xe-select-v1</x:v>
       </x:c>
       <x:c r="O88" s="3" t="str">
-        <x:v>缺段</x:v>
+        <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P88" s="3" t="str">
-        <x:v>演示重建：缺少入营选拔评审记录，未补造评价或评价人。</x:v>
+        <x:v>演示重建：完成了最小主流程；评审时未充分展示边界场景，按原档位记录。</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="48" customHeight="1">
@@ -4521,32 +4453,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D89" s="3" t="str">
-        <x:v>bow-923-work-088</x:v>
+        <x:v>bow-923-v3-work-088</x:v>
       </x:c>
       <x:c r="E89" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F89" s="3"/>
       <x:c r="G89" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H89" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I89" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J89" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>优先录取</x:v>
       </x:c>
       <x:c r="K89" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-17</x:v>
       </x:c>
       <x:c r="L89" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>贺云舒（演示）</x:v>
       </x:c>
       <x:c r="M89" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N89" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -4569,32 +4501,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D90" s="3" t="str">
-        <x:v>bow-923-work-089</x:v>
+        <x:v>bow-923-v3-work-089</x:v>
       </x:c>
       <x:c r="E90" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F90" s="3"/>
       <x:c r="G90" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H90" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I90" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J90" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="K90" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-17</x:v>
       </x:c>
       <x:c r="L90" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>贺云舒（演示）</x:v>
       </x:c>
       <x:c r="M90" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N90" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -4603,7 +4535,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P90" s="3" t="str">
-        <x:v>演示重建：作品主流程完整，能说明一次方案取舍，并现场复现失败后的恢复步骤。</x:v>
+        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="48" customHeight="1">
@@ -4617,32 +4549,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D91" s="3" t="str">
-        <x:v>bow-923-work-090</x:v>
+        <x:v>bow-923-v3-work-090</x:v>
       </x:c>
       <x:c r="E91" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F91" s="3"/>
       <x:c r="G91" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H91" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I91" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J91" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="K91" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-17</x:v>
       </x:c>
       <x:c r="L91" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>贺云舒（演示）</x:v>
       </x:c>
       <x:c r="M91" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N91" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -4651,7 +4583,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P91" s="3" t="str">
-        <x:v>演示重建：作品主流程完整，能说明一次方案取舍，并现场复现失败后的恢复步骤。</x:v>
+        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="48" customHeight="1">
@@ -4665,27 +4597,41 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D92" s="3" t="str">
-        <x:v>bow-923-work-091</x:v>
+        <x:v>bow-923-v3-work-091</x:v>
       </x:c>
       <x:c r="E92" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F92" s="3"/>
-      <x:c r="G92" s="3"/>
-      <x:c r="H92" s="3"/>
-      <x:c r="I92" s="3"/>
-      <x:c r="J92" s="3"/>
-      <x:c r="K92" s="3"/>
-      <x:c r="L92" s="3"/>
-      <x:c r="M92" s="10"/>
+      <x:c r="G92" s="3" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="H92" s="3" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="I92" s="3" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="J92" s="3" t="str">
+        <x:v>优先录取</x:v>
+      </x:c>
+      <x:c r="K92" s="3" t="str">
+        <x:v>s-17</x:v>
+      </x:c>
+      <x:c r="L92" s="3" t="str">
+        <x:v>贺云舒（演示）</x:v>
+      </x:c>
+      <x:c r="M92" s="10" t="n">
+        <x:v>46203.04166666667</x:v>
+      </x:c>
       <x:c r="N92" s="3" t="str">
         <x:v>xe-select-v1</x:v>
       </x:c>
       <x:c r="O92" s="3" t="str">
-        <x:v>缺段</x:v>
+        <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P92" s="3" t="str">
-        <x:v>演示重建：缺少入营选拔评审记录，未补造评价或评价人。</x:v>
+        <x:v>演示重建：作品主流程完整，能说明一次方案取舍，并现场复现失败后的恢复步骤。</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
@@ -4699,32 +4645,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D93" s="3" t="str">
-        <x:v>bow-923-work-092</x:v>
+        <x:v>bow-923-v3-work-092</x:v>
       </x:c>
       <x:c r="E93" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F93" s="3"/>
       <x:c r="G93" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="H93" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I93" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J93" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="K93" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-17</x:v>
       </x:c>
       <x:c r="L93" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>贺云舒（演示）</x:v>
       </x:c>
       <x:c r="M93" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N93" s="3" t="str">
         <x:v>xe-select-v1</x:v>
@@ -4733,7 +4679,7 @@
         <x:v>已确认（演示）</x:v>
       </x:c>
       <x:c r="P93" s="3" t="str">
-        <x:v>演示重建：作品主流程完整，能说明一次方案取舍，并现场复现失败后的恢复步骤。</x:v>
+        <x:v>演示重建：作品可运行，说明了基本实现；异常场景的取舍仍需补充证据。</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="48" customHeight="1">
@@ -4747,32 +4693,32 @@
         <x:v>XEngineer 第六期（演示）</x:v>
       </x:c>
       <x:c r="D94" s="3" t="str">
-        <x:v>bow-923-work-093</x:v>
+        <x:v>bow-923-v3-work-093</x:v>
       </x:c>
       <x:c r="E94" s="3" t="str">
         <x:v>个人作品</x:v>
       </x:c>
       <x:c r="F94" s="3"/>
       <x:c r="G94" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H94" s="3" t="str">
-        <x:v>中间档</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="I94" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="J94" s="3" t="str">
-        <x:v>高分档</x:v>
+        <x:v>优先录取</x:v>
       </x:c>
       <x:c r="K94" s="3" t="str">
-        <x:v>s-04</x:v>
+        <x:v>s-17</x:v>
       </x:c>
       <x:c r="L94" s="3" t="str">
-        <x:v>杜安歌（演示）</x:v>
+        <x:v>贺云舒（演示）</x:v>
       </x:c>
       <x:c r="M94" s="10" t="n">
-        <x:v>46083.04166666667</x:v>
+        <x:v>46203.04166666667</x:v>
       </x:c>
       <x:c r="N94" s="3" t="str">
         <x:v>xe-select-v1</x:v>

</xml_diff>